<commit_message>
excluyendo columnas subject time
</commit_message>
<xml_diff>
--- a/resultados_clasificadores/naive_bayes_modelo1.xlsx
+++ b/resultados_clasificadores/naive_bayes_modelo1.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Priors" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Medias" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Varianzas" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Priors" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Medias" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Varianzas" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -469,61 +469,56 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K3"/>
+  <dimension ref="A1:J3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Time</t>
+          <t>EDA_SCR_count</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>EDA_SCR_count</t>
+          <t>EDA_Phasic_AUC</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>EDA_Phasic_AUC</t>
+          <t>EDA_Tonic_Mean</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>EDA_Tonic_Mean</t>
+          <t>HRV_RMSSD</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>HRV_RMSSD</t>
+          <t>HRV_SDNN</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>HRV_SDNN</t>
+          <t>HRV_MeanNN</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>HRV_MeanNN</t>
+          <t>HRV_LF</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>HRV_LF</t>
+          <t>HRV_HF</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>HRV_HF</t>
+          <t>HRV_LFHF</t>
         </is>
       </c>
       <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>HRV_LFHF</t>
-        </is>
-      </c>
-      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Clase</t>
         </is>
@@ -531,71 +526,65 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>2189.234693877551</v>
+        <v>-0.03852068755220759</v>
       </c>
       <c r="B2" t="n">
-        <v>-0.03852068755220759</v>
+        <v>-0.09596117372763521</v>
       </c>
       <c r="C2" t="n">
-        <v>-0.09596117372763521</v>
+        <v>-0.07413077004900862</v>
       </c>
       <c r="D2" t="n">
-        <v>-0.07413077004900862</v>
+        <v>0.096202645907012</v>
       </c>
       <c r="E2" t="n">
-        <v>0.096202645907012</v>
+        <v>0.09947306525962649</v>
       </c>
       <c r="F2" t="n">
-        <v>0.09947306525962649</v>
+        <v>0.2974099454560232</v>
       </c>
       <c r="G2" t="n">
-        <v>0.2974099454560232</v>
+        <v>-0.01438918003060385</v>
       </c>
       <c r="H2" t="n">
-        <v>-0.01438918003060385</v>
+        <v>0.007807661902554599</v>
       </c>
       <c r="I2" t="n">
-        <v>0.007807661902554599</v>
+        <v>0.0002015166163728263</v>
       </c>
       <c r="J2" t="n">
-        <v>0.0002015166163728263</v>
-      </c>
-      <c r="K2" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>2963.368421052632</v>
+        <v>0.490311701763354</v>
       </c>
       <c r="B3" t="n">
-        <v>0.490311701763354</v>
+        <v>0.3795169194846558</v>
       </c>
       <c r="C3" t="n">
-        <v>0.3795169194846558</v>
+        <v>0.2934017937631542</v>
       </c>
       <c r="D3" t="n">
-        <v>0.2934017937631542</v>
+        <v>-0.4250328589123709</v>
       </c>
       <c r="E3" t="n">
-        <v>-0.4250328589123709</v>
+        <v>-0.472669253778164</v>
       </c>
       <c r="F3" t="n">
-        <v>-0.472669253778164</v>
+        <v>-1.160138601145313</v>
       </c>
       <c r="G3" t="n">
-        <v>-1.160138601145313</v>
+        <v>-0.1378024587391029</v>
       </c>
       <c r="H3" t="n">
-        <v>-0.1378024587391029</v>
+        <v>-0.01235441874431974</v>
       </c>
       <c r="I3" t="n">
-        <v>-0.01235441874431974</v>
+        <v>-0.1561861430528349</v>
       </c>
       <c r="J3" t="n">
-        <v>-0.1561861430528349</v>
-      </c>
-      <c r="K3" t="n">
         <v>1</v>
       </c>
     </row>
@@ -610,61 +599,56 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K3"/>
+  <dimension ref="A1:J3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Time</t>
+          <t>EDA_SCR_count</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>EDA_SCR_count</t>
+          <t>EDA_Phasic_AUC</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>EDA_Phasic_AUC</t>
+          <t>EDA_Tonic_Mean</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>EDA_Tonic_Mean</t>
+          <t>HRV_RMSSD</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>HRV_RMSSD</t>
+          <t>HRV_SDNN</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>HRV_SDNN</t>
+          <t>HRV_MeanNN</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>HRV_MeanNN</t>
+          <t>HRV_LF</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>HRV_LF</t>
+          <t>HRV_HF</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>HRV_HF</t>
+          <t>HRV_LFHF</t>
         </is>
       </c>
       <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>HRV_LFHF</t>
-        </is>
-      </c>
-      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Clase</t>
         </is>
@@ -672,71 +656,65 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>3519807.580580026</v>
+        <v>0.8472000266172246</v>
       </c>
       <c r="B2" t="n">
-        <v>0.8502082062144186</v>
+        <v>0.8837154507145949</v>
       </c>
       <c r="C2" t="n">
-        <v>0.8867236303117889</v>
+        <v>0.9538493277858952</v>
       </c>
       <c r="D2" t="n">
-        <v>0.9568575073830892</v>
+        <v>0.9912280974317764</v>
       </c>
       <c r="E2" t="n">
-        <v>0.9942362770289704</v>
+        <v>0.9871802877712135</v>
       </c>
       <c r="F2" t="n">
-        <v>0.9901884673684075</v>
+        <v>0.6486114974325676</v>
       </c>
       <c r="G2" t="n">
-        <v>0.6516196770297616</v>
+        <v>0.9236086464360825</v>
       </c>
       <c r="H2" t="n">
-        <v>0.9266168260332766</v>
+        <v>0.9761296801391566</v>
       </c>
       <c r="I2" t="n">
-        <v>0.9791378597363506</v>
+        <v>1.084133540810768</v>
       </c>
       <c r="J2" t="n">
-        <v>1.087141720407962</v>
-      </c>
-      <c r="K2" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>414666.5514846349</v>
+        <v>1.232970106079812</v>
       </c>
       <c r="B3" t="n">
-        <v>1.235978285677006</v>
+        <v>1.497733294677502</v>
       </c>
       <c r="C3" t="n">
-        <v>1.500741474274696</v>
+        <v>1.287994219140043</v>
       </c>
       <c r="D3" t="n">
-        <v>1.291002398737237</v>
+        <v>0.9591051360910405</v>
       </c>
       <c r="E3" t="n">
-        <v>0.9621133156882345</v>
+        <v>0.6316859245261384</v>
       </c>
       <c r="F3" t="n">
-        <v>0.6346941041233324</v>
+        <v>0.6988790527465047</v>
       </c>
       <c r="G3" t="n">
-        <v>0.7018872323436988</v>
+        <v>1.139331142695961</v>
       </c>
       <c r="H3" t="n">
-        <v>1.142339322293155</v>
+        <v>1.033375409116194</v>
       </c>
       <c r="I3" t="n">
-        <v>1.036383588713388</v>
+        <v>0.6265394176665279</v>
       </c>
       <c r="J3" t="n">
-        <v>0.6295475972637219</v>
-      </c>
-      <c r="K3" t="n">
         <v>1</v>
       </c>
     </row>

</xml_diff>